<commit_message>
feat(qa): expand QA.xlsx to 105 comprehensive, categorized Q&A pairs covering all student scenarios
</commit_message>
<xml_diff>
--- a/subspaces/01-academic-training/schedule-deadline-agent/agent/QA.xlsx
+++ b/subspaces/01-academic-training/schedule-deadline-agent/agent/QA.xlsx
@@ -50,7 +50,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00004B87"/>
+        <fgColor rgb="00003366"/>
       </patternFill>
     </fill>
     <fill>
@@ -473,14 +473,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -501,7 +501,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Câu trả lời của Agent (Chuẩn hóa)</t>
+          <t>Câu trả lời của Agent (Chuẩn hóa &amp; Chi tiết)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Theo Kế hoạch năm học 2025-2026 của HCMUS, Học kỳ 1 chính thức bắt đầu từ ngày 22/9/2025 đến ngày 05/10/2025 (dự kiến) áp dụng cho cả Khối Chương trình Chuẩn và Chương trình Đề án (Tiên tiến/CLC).</t>
+          <t>Theo Kế hoạch năm học 2025-2026 (dự kiến) của HCMUS, Học kỳ 1 chính thức bắt đầu từ ngày 22/9/2025 đến ngày 05/10/2025 đối với cả Chương trình Chuẩn và Chương trình Đề án.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>HK1, bắt đầu học kỳ, khai giảng, lịch học kỳ 1</t>
+          <t>HK1, bắt đầu kỳ 1, ngày khai giảng, lịch học kỳ 1</t>
         </is>
       </c>
     </row>
@@ -546,19 +546,20 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Tân sinh viên K2025 bắt đầu các hoạt động đầu khóa vào thời gian nào?</t>
+          <t>Lịch trình đầu khóa của tân sinh viên K2025 gồm những mốc nào?</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Tân sinh viên khóa 2025 có hai mốc quan trọng đầu khóa:
-1. Từ 04/9 đến 19/9/2025: Gặp gỡ Ban Chủ nhiệm Khoa và tham gia Tuần sinh hoạt phổ biến quy chế đầu khóa (bắt buộc dự, vắng trừ 20 ĐRL).
-2. Ngày 05/9/2025: Kỳ thi tiếng Anh phân loại đầu khóa K2025.</t>
+          <t>Tân sinh viên K2025 cần lưu ý 3 mốc quan trọng đầu năm:
+1. 04/9 – 19/9/2025: Gặp gỡ Ban Chủ nhiệm Khoa và tham gia Tuần sinh hoạt công dân phổ biến quy chế (bắt buộc, vắng trừ 20 ĐRL).
+2. 05/9/2025: Kỳ thi tiếng Anh phân loại đầu khóa K2025.
+3. 22/9 – 05/10/2025: Chính thức vào học tuần đầu tiên của HK1.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>tân sinh viên, K2025, sinh hoạt đầu khóa, thi tiếng Anh</t>
+          <t>tân sinh viên, K2025, lịch đầu khóa, sinh hoạt công dân</t>
         </is>
       </c>
     </row>
@@ -573,18 +574,19 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Chương trình Chuẩn và Chương trình Đề án khác nhau thế nào về số học kỳ?</t>
+          <t>Một năm học tại HCMUS kéo dài bao nhiêu học kỳ?</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>- Chương trình Chuẩn (đại trà): Gồm 02 học kỳ chính (mỗi kỳ 15 tuần thực học) và 01 Học kỳ Hè tự chọn (ít nhất 5 tuần) để học lại/cải thiện/học vượt.
-- Chương trình Đề án (Tiên tiến, CLC, Liên kết): Gồm 03 học kỳ chính thức liên tục trong năm (tổng tối thiểu 30 tuần lên lớp), không có kỳ hè riêng.</t>
+          <t>Tùy theo hệ đào tạo:
+- Chương trình Chuẩn: Có 02 học kỳ chính (mỗi kỳ 15 tuần thực học) và 01 Học kỳ Hè (ít nhất 5 tuần thực học).
+- Chương trình Đề án (Tiên tiến, CLC, Liên kết): Có 03 học kỳ chính thức liên tục trong năm (tổng tối thiểu 30 tuần lên lớp), không có kỳ hè riêng.</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>chương trình chuẩn, chương trình đề án, số học kỳ, 3 học kỳ</t>
+          <t>số học kỳ, cơ cấu năm học, chương trình chuẩn, chương trình đề án</t>
         </is>
       </c>
     </row>
@@ -605,13 +607,13 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Lịch bắt đầu HK2 khác nhau theo hệ đào tạo:
-- Chương trình Chuẩn: Bắt đầu từ 02/3 – 08/3/2026 (sau kỳ nghỉ Tết).
-- Chương trình Đề án: Bắt đầu từ 12/01 – 18/01/2026 (học trước Tết 1 tuần rồi nghỉ Tết).</t>
+- Khối Chương trình Chuẩn: Bắt đầu từ ngày 02/3/2026 – 08/3/2026 (sau kỳ nghỉ Tết Nguyên Đán).
+- Khối Chương trình Đề án: Bắt đầu sớm từ ngày 12/01/2026 – 18/01/2026 (học trước Tết 1 tuần rồi mới nghỉ Tết).</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>HK2, bắt đầu kỳ 2, thời gian học kỳ 2</t>
+          <t>bắt đầu HK2, học kỳ 2, lịch HK2</t>
         </is>
       </c>
     </row>
@@ -626,20 +628,20 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Học kỳ Hè của năm học 2025-2026 diễn ra vào lúc nào?</t>
+          <t>Học kỳ Hè năm 2026 bắt đầu và kết thúc vào lúc nào?</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Học kỳ Hè chỉ áp dụng cho Chương trình Chuẩn:
-- Bắt đầu học: Từ ngày 20/7/2026 – 26/7/2026.
-- Thi kết thúc học kỳ Hè: Từ ngày 31/8/2026 – 06/9/2026.
-Sinh viên được đăng ký tối đa 12 tín chỉ trong kỳ Hè.</t>
+          <t>Học kỳ Hè (dành riêng cho Chương trình Chuẩn) có lịch như sau:
+- Bắt đầu học kỳ hè: 20/7/2026 – 26/7/2026.
+- Thi kết thúc học phần HK Hè: 31/8/2026 – 06/9/2026.
+Sinh viên được đăng ký tối đa 12 tín chỉ trong học kỳ hè.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>học kỳ hè, kỳ hè, lịch kỳ hè, hè 2026</t>
+          <t>học kỳ hè, kỳ hè 2026, lịch hè, thi hè</t>
         </is>
       </c>
     </row>
@@ -654,20 +656,20 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Chương trình Đề án có học kỳ 3 không và diễn ra khi nào?</t>
+          <t>Học kỳ 3 của Chương trình Đề án diễn ra vào thời gian nào?</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Có. Chương trình Đề án vận hành Học kỳ 3 như một kỳ chính thức:
-- Bắt đầu HK3: 18/5 – 24/5/2026.
-- Thi giữa HK3: 29/6 – 05/7/2026.
-- Thi kết thúc HK3: 10/8 – 23/8/2026.</t>
+          <t>Học kỳ 3 (chương trình chính khóa của khối Đề án) có lịch trình:
+- Bắt đầu HK3: 18/5/2026 – 24/5/2026.
+- Thi giữa HK3: 29/6/2026 – 05/7/2026.
+- Thi kết thúc HK3: 10/8/2026 – 23/8/2026.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>học kỳ 3, HK3, đề án, lịch HK3</t>
+          <t>học kỳ 3, HK3, khối đề án, lịch HK3</t>
         </is>
       </c>
     </row>
@@ -677,24 +679,26 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Lịch thi cử</t>
+          <t>Kế hoạch năm học</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Lịch thi giữa học kỳ 1 năm học 2025-2026 là ngày nào?</t>
+          <t>Thời gian tối đa để hoàn thành khóa học đại học tại HCMUS là bao lâu?</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Lịch thi giữa HK1 phân biệt rõ giữa hai chương trình:
-- Chương trình Đề án: Thi giữa kỳ từ 10/11/2025 đến 16/11/2025.
-- Chương trình Chuẩn: Thi giữa kỳ từ 24/11/2025 đến 30/11/2025 (sau khối Đề án 2 tuần).</t>
+          <t>Theo Khoản 7 Điều 2 Quy chế Đào tạo (QĐ 1175/QĐ-KHTN):
+- Sinh viên được rút ngắn tối đa 01 năm hoặc kéo dài không quá 03 năm học so với kế hoạch 4 năm (tổng tối đa là 7 năm).
+- Không vượt quá 2 lần thời gian thiết kế của khóa học.
+- Chương trình liên thông: kéo dài không quá 02 năm.
+- Quá thời hạn tối đa này, sinh viên sẽ bị xóa tên khỏi danh sách Trường.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>thi giữa kỳ, midterm, thi giữa kỳ 1, lịch thi</t>
+          <t>thời gian tối đa, hoàn thành khóa học, kéo dài thời gian, quá hạn học tập</t>
         </is>
       </c>
     </row>
@@ -704,23 +708,22 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Lịch thi cử</t>
+          <t>Kế hoạch năm học</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Khi nào thi cuối học kỳ 1 năm học 2025-2026?</t>
+          <t>Sinh viên có thể học vượt để tốt nghiệp sớm bao nhiêu năm?</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>- Chương trình Đề án: Thi kết thúc học phần HK1 từ 22/12/2025 đến 04/01/2026 (thi xong trước Tết Dương lịch và Nguyên đán).
-- Chương trình Chuẩn: Thi kết thúc học phần HK1 từ 19/01/2026 đến 08/02/2026.</t>
+          <t>Theo Điểm a Khoản 7 Điều 2 Quy chế Đào tạo, sinh viên có học lực tốt được phép chủ động đăng ký học vượt và rút ngắn tối đa 01 năm học so với kế hoạch đào tạo chuẩn (hoàn thành chương trình trong 3 năm).</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>thi cuối kỳ, final exam, thi HK1, thi kết thúc học phần</t>
+          <t>học vượt, tốt nghiệp sớm, rút ngắn thời gian</t>
         </is>
       </c>
     </row>
@@ -730,23 +733,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Lịch thi cử</t>
+          <t>Kế hoạch năm học</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Lịch thi giữa học kỳ 2 và cuối học kỳ 2 là khi nào?</t>
+          <t>Một năm học sinh viên tích lũy trung bình bao nhiêu tín chỉ theo kế hoạch chuẩn?</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>- Chương trình Chuẩn: Thi giữa HK2 từ 04/5 – 10/5/2026; Thi cuối HK2 từ 29/6 – 19/7/2026.
-- Chương trình Đề án: Thi giữa HK2 từ 16/3 – 22/3/2026; Thi cuối HK2 từ 27/4 – 10/5/2026.</t>
+          <t>Theo Khoản 3 Điều 15 Quy chế Đào tạo, số tín chỉ trung bình một năm học theo kế hoạch học tập chuẩn của Trường là 38 tín chỉ.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>thi HK2, thi giữa kỳ 2, thi cuối kỳ 2</t>
+          <t>tín chỉ một năm, tiến độ chuẩn, 38 tín chỉ</t>
         </is>
       </c>
     </row>
@@ -756,22 +758,26 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Lịch thi cử</t>
+          <t>Kế hoạch năm học</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Đến phòng thi trễ bao nhiêu phút thì không được vào thi?</t>
+          <t>Xếp trình độ năm học (năm 1, 2, 3, 4) được tính dựa trên số tín chỉ nào?</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Theo quy chế khảo thí của Trường, sinh viên đến chậm quá 15 PHÚT sau khi đề thi đã được phát sẽ TUYỆT ĐỐI KHÔNG ĐƯỢC VÀO PHÒNG THI và bị tính là vắng thi không phép (nhận điểm 0).</t>
+          <t>Căn cứ Khoản 3 Điều 15 Quy chế Đào tạo:
+- Trình độ năm 1: Tích lũy N &lt; 38 tín chỉ.
+- Trình độ năm 2: 38 &lt;= N &lt; 76 tín chỉ.
+- Trình độ năm 3: 76 &lt;= N &lt; 114 tín chỉ.
+- Trình độ năm 4: N &gt;= 114 tín chỉ.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>trễ giờ thi, đi muộn, quy định phòng thi, 15 phút</t>
+          <t>xếp năm học, sinh viên năm 2, sinh viên năm 3, tích lũy tín chỉ</t>
         </is>
       </c>
     </row>
@@ -786,17 +792,18 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Tôi cần mang giấy tờ gì khi vào phòng thi?</t>
+          <t>Lịch thi giữa học kỳ 1 (Midterm) của năm học 2025-2026 là ngày nào?</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Sinh viên bắt buộc phải xuất trình Thẻ Sinh viên còn hiệu lực. Trong trường hợp mất thẻ SV, sinh viên phải mang Căn cước công dân (CCCD) gắn chip kèm theo Giấy xác nhận sinh viên do Phòng CTSV cấp.</t>
+          <t>- Chương trình Đề án (Tiên tiến/CLC): Thi giữa HK1 từ ngày 10/11/2025 đến ngày 16/11/2025.
+- Chương trình Chuẩn (Đại trà): Thi giữa HK1 từ ngày 24/11/2025 đến ngày 30/11/2025 (sau khối Đề án 2 tuần).</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>giấy tờ phòng thi, thẻ sinh viên, CCCD, mất thẻ</t>
+          <t>thi giữa kỳ 1, midterm HK1, lịch thi giữa kỳ</t>
         </is>
       </c>
     </row>
@@ -806,24 +813,23 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Lịch nghỉ Tết</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Trường ĐH Khoa học Tự nhiên nghỉ Tết Nguyên Đán 2026 bao lâu?</t>
+          <t>Lịch thi kết thúc học phần (Final Exam) Học kỳ 1 là khi nào?</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Lịch nghỉ Tết có sự khác biệt giữa hai hệ đào tạo:
-- Chương trình Chuẩn: Khung thời gian từ 19/01/2026 đến 08/02/2026 (trùng thời gian thi HK1; sinh viên thi xong môn cuối cùng của mình là bắt đầu được nghỉ Tết).
-- Chương trình Đề án: Nghỉ trọn vẹn từ 09/02/2026 đến 01/3/2026 (sau khi đã hoàn tất thi HK1 và học tuần đầu HK2).</t>
+          <t>- Chương trình Đề án: Thi cuối HK1 từ 22/12/2025 đến 04/01/2026 (thi xong hoàn toàn trước Tết Dương lịch &amp; Tết Nguyên đán).
+- Chương trình Chuẩn: Thi cuối HK1 từ 19/01/2026 đến 08/02/2026 (khung thời gian thi trùng với dịp giáp Tết).</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>nghỉ tết, tết nguyên đán, tết 2026, lịch nghỉ tết</t>
+          <t>thi cuối kỳ 1, thi kết thúc học phần HK1, final exam</t>
         </is>
       </c>
     </row>
@@ -833,22 +839,23 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Deadline Hồ sơ</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Hạn chót nộp hồ sơ Miễn giảm học phí học kỳ 1 là khi nào?</t>
+          <t>Lịch thi giữa kỳ và cuối kỳ của Học kỳ 2 là những ngày nào?</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Hạn chót nộp hồ sơ Miễn giảm học phí (MGHP), Trợ cấp xã hội (TCXH) và các Chế độ chính sách cho HK1 là từ ngày 22/9/2025 đến hết ngày 03/10/2025. Hồ sơ nộp trực tiếp tại Phòng Công tác Sinh viên (P. A02 CS1 hoặc 2.8 CS2). Sau ngày 03/10 Nhà trường không nhận bổ sung.</t>
+          <t>- Chương trình Chuẩn: Thi giữa HK2 từ 04/5 – 10/5/2026; Thi cuối HK2 từ 29/6 – 19/7/2026.
+- Chương trình Đề án: Thi giữa HK2 từ 16/3 – 22/3/2026; Thi cuối HK2 từ 27/4 – 10/5/2026.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>miễn giảm học phí, MGHP, TCXH, hạn nộp hồ sơ HK1</t>
+          <t>thi giữa kỳ 2, thi cuối kỳ 2, lịch thi HK2</t>
         </is>
       </c>
     </row>
@@ -858,22 +865,23 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Deadline Hồ sơ</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Nếu tôi nộp hồ sơ miễn giảm học phí trễ hạn thì sao?</t>
+          <t>Lịch thi kết thúc học phần Học kỳ Hè và Học kỳ 3 là khi nào?</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Nếu nộp trễ sau hạn 03/10/2025, bạn sẽ KHÔNG ĐƯỢC GIẢI QUYẾT miễn giảm trong HK1. Bạn bắt buộc phải đóng đủ 100% học phí đúng hạn để không bị buộc thôi học, sau đó chờ đến đợt nộp HK2 (02/3 – 15/3/2026) để nộp lại.</t>
+          <t>- Thi Học kỳ Hè (Khối Chuẩn): Từ ngày 31/8/2026 đến ngày 06/9/2026.
+- Thi Học kỳ 3 (Khối Đề án): Thi giữa HK3 từ 29/6 – 05/7/2026; Thi cuối HK3 từ 10/8 – 23/8/2026.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>trễ hạn MGHP, muộn nộp hồ sơ, hậu quả trễ hạn</t>
+          <t>thi hè, thi HK3, lịch thi học kỳ 3</t>
         </is>
       </c>
     </row>
@@ -883,22 +891,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Deadline Hồ sơ</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Hạn nộp hồ sơ miễn giảm học phí cho học kỳ 2 là ngày nào?</t>
+          <t>Đi thi muộn bao nhiêu phút thì bị cấm vào phòng thi?</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Thời gian nhận hồ sơ MGHP và TCXH cho Học kỳ 2 là từ ngày 02/3/2026 đến ngày 15/3/2026 tại Phòng Công tác Sinh viên.</t>
+          <t>Theo Quy chế Khảo thí của Trường, sinh viên đến chậm quá 15 PHÚT sau khi đề thi đã được phát sẽ TUYỆT ĐỐI KHÔNG ĐƯỢC VÀO PHÒNG THI và bị tính là vắng thi không phép (nhận điểm 0).</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>hạn nộp MGHP kỳ 2, deadline kỳ 2</t>
+          <t>trễ giờ thi, đi muộn 15 phút, cấm thi, vắng thi</t>
         </is>
       </c>
     </row>
@@ -908,22 +916,22 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Deadline Ngoại trú</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Thời hạn xác nhận ngoại trú học kỳ 1 là khi nào và làm ở đâu?</t>
+          <t>Vào phòng thi cần xuất trình giấy tờ gì?</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Thời gian xác nhận thông tin ngoại trú HK1 là từ ngày 27/10/2025 đến ngày 07/11/2025. Sinh viên thực hiện khai báo trực tuyến trên hệ thống quản lý sinh viên hoặc nộp Giấy xác nhận tạm trú về Phòng CTSV.</t>
+          <t>Sinh viên bắt buộc phải xuất trình Thẻ Sinh viên còn hiệu lực. Nếu mất thẻ SV, sinh viên phải mang theo Căn cước công dân (CCCD) gắn chip còn hạn kèm theo Giấy xác nhận sinh viên do Phòng CTSV cấp.</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>ngoại trú, xác nhận ngoại trú, hạn ngoại trú HK1</t>
+          <t>thẻ sinh viên, giấy tờ phòng thi, CCCD, mất thẻ sinh viên</t>
         </is>
       </c>
     </row>
@@ -933,22 +941,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Deadline Ngoại trú</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Không xác nhận ngoại trú đúng hạn có bị phạt không?</t>
+          <t>Đem điện thoại vào phòng thi có bị lập biên bản không?</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>CÓ. Theo Quy chế Đánh giá kết quả rèn luyện của Trường, sinh viên không xác nhận ngoại trú đúng thời hạn sẽ BỊ TRỪ 15 ĐIỂM RÈN LUYỆN trong học kỳ đó. Mức trừ này làm bạn bị hạ bậc xếp loại rèn luyện và mất cơ hội xét học bổng.</t>
+          <t>CÓ. Theo Quy định Khảo thí, sinh viên tuyệt đối không được mang điện thoại di động, đồng hồ thông minh hoặc thiết bị truyền thông vào chỗ ngồi thi (kể cả khi đã tắt nguồn). Vi phạm sẽ bị lập biên bản đình chỉ thi và nhận điểm 0.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>trừ điểm ngoại trú, phạt ngoại trú, 15 điểm</t>
+          <t>mang điện thoại phòng thi, gian lận, kỷ luật phòng thi</t>
         </is>
       </c>
     </row>
@@ -958,24 +966,22 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Điểm rèn luyện</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Thời gian đánh giá điểm rèn luyện diễn ra vào lúc nào?</t>
+          <t>Mức kỷ luật phòng thi: Khiển trách bị trừ bao nhiêu phần trăm điểm?</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>- Đánh giá HK1: Tháng 01/2026 đến tháng 03/2026.
-- Đánh giá HK2: Tháng 07/2026 – 10/2026 (Khối Chuẩn); Tháng 05/2026 – 07/2026 (Khối Đề án).
-- Đánh giá HK3: Tháng 09/2026 – 10/2026 (Khối Đề án).</t>
+          <t>Theo Quy định Khảo thí, sinh viên bị xử lý kỷ luật mức Khiển trách sẽ BỊ TRỪ 25% ĐIỂM của bài thi học phần đó.</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>đánh giá điểm rèn luyện, ĐRL, thời gian chấm rèn luyện</t>
+          <t>khiển trách thi, trừ điểm, trừ 25% điểm</t>
         </is>
       </c>
     </row>
@@ -985,23 +991,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Điểm rèn luyện</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Không tham gia Tuần sinh hoạt công dân đầu năm bị phạt thế nào?</t>
+          <t>Mức kỷ luật Cảnh cáo phòng thi bị xử lý thế nào?</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>- Vắng mặt không lý do đầy đủ trong tuần sinh hoạt công dân: BỊ TRỪ 20 ĐIỂM RÈN LUYỆN/đợt.
-- Không nộp bài thu hoạch sau tuần sinh hoạt: BỊ TRỪ 10 ĐIỂM RÈN LUYỆN/đợt.</t>
+          <t>Sinh viên bị kỷ luật mức Cảnh cáo trong ca thi sẽ BỊ TRỪ 50% ĐIỂM của bài thi học phần đó.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>sinh hoạt công dân, trừ điểm công dân, bài thu hoạch</t>
+          <t>cảnh cáo phòng thi, trừ 50% điểm</t>
         </is>
       </c>
     </row>
@@ -1011,22 +1016,22 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Tiết học &amp; Giờ học</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Tiết 1 buổi sáng ở Cơ sở 227 Nguyễn Văn Cừ bắt đầu lúc mấy giờ?</t>
+          <t>Đình chỉ thi trong ca thi bị xử lý thế nào?</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Tại Cơ sở 1 (227 Nguyễn Văn Cừ, Q.5), Tiết 1 buổi sáng bắt đầu lúc 06g40 và kết thúc lúc 07g30. Tiết 2 từ 07g30 đến 08g20.</t>
+          <t>Sinh viên bị kỷ luật mức Đình chỉ thi sẽ BỊ NHẬN ĐIỂM 0 (không điểm) cho học phần đó và không được tiếp tục làm bài thi.</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>tiết 1, giờ học cơ sở 1, Nguyễn Văn Cừ, 6h40</t>
+          <t>đình chỉ thi, nhận điểm 0</t>
         </is>
       </c>
     </row>
@@ -1036,24 +1041,24 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Tiết học &amp; Giờ học</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Giờ học ở Cơ sở Linh Trung (Cơ sở 2) khác Cơ sở 1 thế nào?</t>
+          <t>Hành vi thi hộ hoặc nhờ người thi hộ bị xử lý kỷ luật thế nào?</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Tại Cơ sở 2 (Khu Đô thị ĐHQG-HCM, Thủ Đức):
-- Tiết 1 sáng bắt đầu lúc 07g30 (muộn hơn Cơ sở 1 là 50 phút).
-- Không có ca học buổi tối (chỉ học từ tiết 1 đến tiết 10, kết thúc lúc 17g00).</t>
+          <t>Hành vi thi hộ hoặc nhờ người thi hộ là vi phạm đặc biệt nghiêm trọng:
+- Vi phạm lần 1: ĐÌNH CHỈ HỌC TẬP 01 NĂM HỌC.
+- Vi phạm lần 2: BUỘC THÔI HỌC VÀ XÓA TÊN KHỎI DANH SÁCH SINH VIÊN TRƯỜNG.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>cơ sở 2, Linh Trung, giờ học, tiết 1 thủ đức</t>
+          <t>thi hộ, nhờ thi hộ, đình chỉ 1 năm, buộc thôi học</t>
         </is>
       </c>
     </row>
@@ -1063,25 +1068,25 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Tiết học &amp; Giờ học</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Ca tối ở Cơ sở 1 gồm những tiết nào, từ mấy giờ?</t>
+          <t>Thời gian làm bài thi kết thúc học phần được quy định bao nhiêu phút?</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Ca tối tại Cơ sở 1 gồm 3 tiết:
-- Tiết 13: 18g00 – 18g50
-- Tiết 14: 18g50 – 19g40
-- Tiết 15: 19g40 – 20g30.</t>
+          <t>Theo Khoản 1 Điều 9 Quy chế Đào tạo:
+- Học phần 1 – 2 tín chỉ: Thời gian thi từ 45 đến 60 phút.
+- Học phần 3 tín chỉ: Thời gian thi từ 60 đến 90 phút.
+- Học phần từ 4 tín chỉ trở lên: Thời gian thi từ 60 đến 120 phút.</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>ca tối, học buổi tối, tiết 13, tiết 14, tiết 15</t>
+          <t>thời gian làm bài thi, bao nhiêu phút, số tín chỉ bài thi</t>
         </is>
       </c>
     </row>
@@ -1091,22 +1096,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Tiết học &amp; Giờ học</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Thời gian nghỉ trưa giữa ca sáng và ca chiều là bao lâu?</t>
+          <t>Tỷ trọng điểm thi cuối kỳ chiếm tối thiểu bao nhiêu phần trăm điểm môn học?</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Ca sáng kết thúc lúc 12g00 (hết tiết 6 ở CS1, hết tiết 5 ở CS2). Ca chiều bắt đầu lúc 12g30 (tiết 7 ở CS1, tiết 6 ở CS2). Khoảng cách nghỉ trưa là đúng 30 phút.</t>
+          <t>Theo Điều 9 Quy chế Đào tạo, điểm thi kết thúc học phần chiếm tỷ trọng KHÔNG DƯỚI 40% (điểm quá trình chiếm từ 50% đến 60% và bao gồm tối thiểu 3 hình thức đánh giá).</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>nghỉ trưa, chuyển ca, ca chiều bắt đầu</t>
+          <t>tỷ trọng điểm thi, điểm quá trình, điểm cuối kỳ, 40%</t>
         </is>
       </c>
     </row>
@@ -1116,23 +1121,22 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Đăng ký học phần</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Sinh viên hệ chuẩn phải đăng ký tối thiểu và tối đa bao nhiêu tín chỉ 1 kỳ?</t>
+          <t>Lịch thi cuối kỳ do phòng ban nào ban hành và xem ở đâu?</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>- Tối thiểu: 14 tín chỉ trong học kỳ chính (không tính GDQP, GDTC và Ngoại ngữ tổng quát).
-- Tối đa: 25 tín chỉ trong học kỳ chính; tối đa 12 tín chỉ trong học kỳ Hè.</t>
+          <t>Lịch thi do Phòng Khảo thí và Đảm bảo Chất lượng (P. KT&amp;ĐBCL) lập và công bố. Sinh viên xem trực tiếp trên Cổng Portal Đào tạo (https://portal.hcmus.edu.vn) hoặc trang web Khảo thí (https://ktdbcl.hcmus.edu.vn).</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>tín chỉ tối thiểu, tín chỉ tối đa, số tín chỉ đăng ký</t>
+          <t>xem lịch thi, phòng khảo thí, tra cứu lịch thi</t>
         </is>
       </c>
     </row>
@@ -1142,24 +1146,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Đăng ký học phần</t>
+          <t>Lịch thi cử</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Chương trình Đề án (CLC/Tiên tiến) quy định số tín chỉ thế nào?</t>
+          <t>Nếu phát hiện bị trùng lịch thi giữa 2 môn thì xử lý thế nào?</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Sinh viên Chương trình Đề án được đăng ký:
-- Tối thiểu: 10 tín chỉ/học kỳ chính.
-- Tối đa: 22 tín chỉ/học kỳ chính.</t>
+          <t>Ngay khi Phòng Khảo thí công bố lịch thi dự kiến, sinh viên phải làm Đơn đề nghị điều chỉnh lịch thi nộp trực tiếp tại Phòng B.04 Cơ sở 1 hoặc gửi email về khaothi@hcmus.edu.vn trước ngày thi ít nhất 07 ngày làm việc để được xếp phòng thi dự phòng.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>tín chỉ chương trình đề án, CLC bao nhiêu tín chỉ</t>
+          <t>trùng lịch thi, điều chỉnh ca thi, xử lý trùng lịch thi</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1171,22 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Đăng ký học phần</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Nếu tôi đăng ký học phần rồi nhưng không đi học thì có sao không?</t>
+          <t>Lịch nghỉ Tết Nguyên Đán 2026 của sinh viên Chương trình Chuẩn là khi nào?</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Sinh viên đã đăng ký học phần mà tự ý không đi học, không kiểm tra sẽ nhận ĐIỂM 0 cho học phần đó. Nếu tự ý bỏ học từ 1 học kỳ chính trở lên sẽ bị Nhà trường BUỘC THÔI HỌC theo quy chế.</t>
+          <t>Theo kế hoạch đào tạo, khung nghỉ Tết của khối Chuẩn bắt đầu từ ngày 19/01/2026 đến ngày 08/02/2026 (trùng khung thời gian thi HK1; sinh viên thi xong môn cuối là được về quê nghỉ Tết).</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>bỏ học, không đi học sau đăng ký, điểm 0, buộc thôi học</t>
+          <t>nghỉ Tết khối chuẩn, Tết Nguyên đán 2026, lịch nghỉ Tết</t>
         </is>
       </c>
     </row>
@@ -1194,25 +1196,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Hoãn thi &amp; Phúc khảo</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Làm sao để xin hoãn thi cuối kỳ khi bị ốm hoặc tai nạn?</t>
+          <t>Lịch nghỉ Tết Nguyên Đán 2026 của sinh viên Chương trình Đề án là khi nào?</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Bạn phải làm thủ tục hoãn thi để nhận điểm I:
-1. Điều kiện: Phải hoàn tất học phí học kỳ đó và có hồ sơ bệnh án/giấy nhập viện hợp lệ từ cấp Quận/Huyện trở lên.
-2. Thời hạn nộp: TRONG VÒNG 05 NGÀY LÀM VIỆC kể từ ngày thi.
-3. Nơi nộp: Phòng Đào tạo (P. B.02 CS1 / P. 2.4 CS2).</t>
+          <t>Sinh viên khối Đề án nghỉ Tết trọn vẹn 3 tuần từ ngày 09/02/2026 đến hết ngày 01/3/2026 (sau khi đã hoàn tất thi HK1 và học tuần đầu của HK2).</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>hoãn thi, điểm I, thủ tục hoãn thi, 5 ngày làm việc</t>
+          <t>nghỉ Tết khối đề án, Tết CLC, 09/02 đến 01/3</t>
         </is>
       </c>
     </row>
@@ -1222,22 +1221,22 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Hoãn thi &amp; Phúc khảo</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Môn được điểm I có phải đóng tiền học lại không?</t>
+          <t>Vì sao lịch nghỉ Tết của 2 chương trình lại lệch nhau?</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>KHÔNG. Sinh viên được cấp điểm I sẽ đăng ký học lại học phần đó trong vòng 01 năm học tiếp theo và KHÔNG PHẢI ĐÓNG LẠI HỌC PHÍ. Tuy nhiên, điểm quá trình sẽ không được bảo lưu mà phải làm lại từ đầu.</t>
+          <t>Do Chương trình Đề án tổ chức 3 học kỳ chính/năm nên tiến độ đẩy sớm: thi HK1 kết thúc trước ngày 04/01/2026, tuần 12/01 – 18/01/2026 bắt đầu HK2 rồi mới nghỉ Tết. Chương trình Chuẩn duy trì 2 kỳ chính nên thi HK1 kéo dài đến giáp Tết.</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>điểm I có đóng học phí không, học lại điểm I</t>
+          <t>vì sao lệch lịch Tết, so sánh lịch nghỉ Tết</t>
         </is>
       </c>
     </row>
@@ -1247,22 +1246,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Hoãn thi &amp; Phúc khảo</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Thời hạn nộp đơn phúc khảo bài thi là bao lâu và nộp ở đâu?</t>
+          <t>Tuần sinh hoạt công dân đầu khóa dành cho ai và diễn ra khi nào?</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Đơn phúc khảo nộp tại Phòng Khảo thí &amp; ĐBCL (Phòng B.04 CS1 / Phòng 2.5 CS2) trong thời hạn quy định sau khi công bố điểm (thường từ 7 – 10 ngày). Kết quả được trả trong vòng 15 ngày làm việc kể từ ngày hết hạn nhận đơn.</t>
+          <t>Diễn ra từ ngày 04/9 đến ngày 19/9/2025, dành cho toàn bộ tân sinh viên khóa 2025. Đây là đợt sinh hoạt bắt buộc để phổ biến quy chế, phương pháp học đại học và gặp gỡ Ban Chủ nhiệm Khoa.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>phúc khảo, nộp đơn phúc khảo, phòng khảo thí, 15 ngày</t>
+          <t>tuần sinh hoạt công dân, đầu khóa, tân sinh viên K2025</t>
         </is>
       </c>
     </row>
@@ -1272,22 +1271,22 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Học phí &amp; Học bổng</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Quá hạn đóng học phí bao lâu thì bị buộc thôi học?</t>
+          <t>Vắng mặt trong Tuần sinh hoạt công dân đầu năm bị phạt thế nào?</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Theo Khoản 2 Điều 16 Quy chế Đào tạo, sinh viên không hoàn thành nghĩa vụ học phí đúng thời hạn thông báo của Trường sẽ bị BUỘC THÔI HỌC và xóa tên khỏi danh sách sinh viên. Nếu gặp khó khăn, bạn phải làm đơn xin gia hạn trước ngày chót.</t>
+          <t>Theo Quy chế Đánh giá kết quả rèn luyện, sinh viên vắng mặt không lý do chính đáng trong Tuần sinh hoạt công dân sẽ BỊ TRỪ 20 ĐIỂM RÈN LUYỆN/đợt.</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>nợ học phí, trễ hạn đóng học phí, buộc thôi học học phí</t>
+          <t>vắng sinh hoạt công dân, trừ 20 điểm rèn luyện, phạt vắng SHCD</t>
         </is>
       </c>
     </row>
@@ -1297,22 +1296,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Học phí &amp; Học bổng</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Thời gian xét học bổng tài trợ doanh nghiệp là khi nào?</t>
+          <t>Không làm bài thu hoạch sau Tuần sinh hoạt công dân bị trừ mấy điểm rèn luyện?</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Các chương trình học bổng tài trợ, học bổng doanh nghiệp, cựu sinh viên thường được thông báo và xét duyệt từ tháng 9 đến tháng 12 năm 2025. Sinh viên theo dõi fanpage và website của Phòng CTSV để chuẩn bị hồ sơ ứng tuyển.</t>
+          <t>Sinh viên không nộp hoặc không hoàn thành bài thu hoạch sau đợt học sinh hoạt công dân sẽ BỊ TRỪ 10 ĐIỂM RÈN LUYỆN/đợt.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>học bổng tài trợ, thời gian xét học bổng, tháng 9 đến tháng 12</t>
+          <t>bài thu hoạch, trừ 10 điểm rèn luyện, không nộp bài thu hoạch</t>
         </is>
       </c>
     </row>
@@ -1322,26 +1321,23 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Phòng ban liên hệ</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Tôi cần xin giấy xác nhận sinh viên hoặc hoãn nghĩa vụ quân sự thì liên hệ phòng nào?</t>
+          <t>Học kỳ 1 năm học kết thúc trước Tết hay sau Tết?</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Liên hệ Phòng Công tác Sinh viên (P. CTSV):
-- Cơ sở 1: Phòng A.02 (227 Nguyễn Văn Cừ, Q.5)
-- Cơ sở 2: Phòng 2.8, Tầng 2 Tòa nhà Điều hành (Thủ Đức)
-- Hotline: 0968 918 018 (Phím 1)
-- Email: congtacsinhvien@hcmus.edu.vn.</t>
+          <t>- Chương trình Đề án: Kết thúc toàn bộ thi HK1 trước Tết (xong ngày 04/01/2026).
+- Chương trình Chuẩn: Thi kết thúc HK1 sát kỳ nghỉ Tết (19/01 – 08/02/2026).</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>giấy xác nhận sinh viên, nghĩa vụ quân sự, phòng CTSV, A.02</t>
+          <t>kết thúc học kỳ 1, trước tết hay sau tết</t>
         </is>
       </c>
     </row>
@@ -1351,26 +1347,22 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Phòng ban liên hệ</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Muốn hỏi về đăng ký môn học và thời khóa biểu thì gặp ai?</t>
+          <t>Thời gian đánh giá điểm rèn luyện Học kỳ 1 diễn ra vào lúc nào?</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Liên hệ Phòng Đào tạo (P. ĐT):
-- Cơ sở 1: Phòng B.02 (227 Nguyễn Văn Cừ, Q.5)
-- Cơ sở 2: Phòng 2.4, Tầng 2 Tòa nhà Điều hành
-- Điện thoại: (028) 62884499 (ext 1200)
-- Email: pdt_khtn@hcmus.edu.vn.</t>
+          <t>Đánh giá kết quả rèn luyện HK1 diễn ra từ tháng 01/2026 đến tháng 03/2026 thông qua 4 cấp: Cá nhân tự chấm -&gt; Ban cán sự lớp họp -&gt; Khoa xét -&gt; Hội đồng cấp Trường phê duyệt.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>phòng đào tạo, đăng ký môn học, B.02, liên hệ phòng đào tạo</t>
+          <t>đánh giá rèn luyện HK1, thời gian chấm rèn luyện</t>
         </is>
       </c>
     </row>
@@ -1380,24 +1372,23 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Phòng ban liên hệ</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Phòng Khảo thí và Đảm bảo Chất lượng nằm ở đâu?</t>
+          <t>Thời gian đánh giá điểm rèn luyện Học kỳ 2 và Học kỳ 3 là khi nào?</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>- Cơ sở 1: Phòng B.04, số 227 Nguyễn Văn Cừ, Quận 5
-- Cơ sở 2: Phòng 2.5, Tầng 2 Tòa nhà Điều hành, Khu ĐT ĐHQG-HCM
-- Email: khaothi@hcmus.edu.vn | Hotline: (028) 62884499 (ext 3370, 3371).</t>
+          <t>- Đánh giá HK2: Tháng 7 – 10/2026 (Khối Chuẩn); Tháng 5 – 07/2026 (Khối Đề án).
+- Đánh giá HK3 (Khối Đề án): Tháng 9 – 10/2026.</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>phòng khảo thí, B.04, phòng thi, liên hệ khảo thí</t>
+          <t>đánh giá rèn luyện HK2, đánh giá rèn luyện HK3</t>
         </is>
       </c>
     </row>
@@ -1407,27 +1398,1794 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Tình huống khẩn cấp</t>
+          <t>Nghỉ Tết &amp; Sinh hoạt</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Tôi gặp khủng hoảng tinh thần và áp lực deadline nặng nề thì có nơi nào hỗ trợ miễn phí không?</t>
+          <t>Ai là người chủ trì việc đánh giá điểm rèn luyện ở cấp lớp?</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Nhà trường có Bộ phận Tham vấn Tâm lý (PSY.US) trực thuộc Phòng CTSV hỗ trợ hoàn toàn miễn phí và bảo mật:
-- Cơ sở 1: Phòng F106A (Dãy F)
-- Cơ sở 2: Phòng C110 (Dãy C)
-- Hotline/Zalo: 0918.207.126 – 0366.812.741
-- Email: hotrosuckhoetinhthan@hcmus.edu.vn
-- Giờ làm việc: Thứ Hai – Thứ Sáu (8g00 – 11g30; 13g30 – 16g30).</t>
+          <t>Ban Cán sự lớp phối hợp cùng Ban Chấp hành Chi đoàn lớp tổ chức cuộc họp toàn thể lớp để xem xét, biểu quyết điểm tự đánh giá của từng sinh viên.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>tham vấn tâm lý, PSY.US, căng thẳng, stress, F106A, trầm cảm</t>
+          <t>họp lớp điểm rèn luyện, ban cán sự, chi đoàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="55" customHeight="1">
+      <c r="A37" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Hạn chót nộp hồ sơ Miễn giảm học phí (MGHP) Học kỳ 1 là ngày nào?</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Hạn chót nộp hồ sơ MGHP, Trợ cấp xã hội (TCXH) và Chế độ chính sách HK1 năm học 2025-2026 là từ ngày 22/9/2025 đến hết ngày 03/10/2025 tại Phòng Công tác Sinh viên (P. A02 CS1 / P. 2.8 CS2).</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>hạn nộp MGHP HK1, deadline miễn giảm học phí, 03/10/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Hạn nộp hồ sơ Miễn giảm học phí Học kỳ 2 là ngày nào?</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Thời hạn tiếp nhận hồ sơ MGHP và TCXH cho Học kỳ 2 là từ ngày 02/3/2026 đến hết ngày 15/3/2026.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>hạn nộp MGHP HK2, deadline học kỳ 2, 15/3/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="55" customHeight="1">
+      <c r="A39" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Nộp hồ sơ miễn giảm học phí ở đâu tại 2 cơ sở?</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>- Cơ sở 1: Phòng A.02, dãy nhà A, số 227 Nguyễn Văn Cừ, Quận 5.
+- Cơ sở 2: Phòng 2.8, Tầng 2 Tòa nhà Điều hành, Khu Đô thị ĐHQG-HCM, Thủ Đức.
+Hotline hỗ trợ: 0968 918 018 (Phím 1).</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>địa chỉ nộp MGHP, nộp hồ sơ ở đâu, phòng A.02, phòng 2.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Nếu tôi nộp hồ sơ miễn giảm học phí sau ngày 03/10/2025 thì có được giải quyết không?</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>TUYỆT ĐỐI KHÔNG. Nhà trường quy định hạn chót hồ sơ MGHP là hạn cứng. Sinh viên nộp trễ sẽ bị hủy quyền lợi trong học kỳ đó, bắt buộc phải đóng đủ 100% học phí và phải chờ đến đợt nộp HK2 (tháng 3/2026) mới được nộp lại.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>nộp trễ MGHP, muộn hồ sơ, có được giải quyết không</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="55" customHeight="1">
+      <c r="A41" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Những đối tượng nào được miễn 100% học phí theo Nghị định 81/2021/NĐ-CP?</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Các nhóm được miễn 100% gồm:
+1. Con người có công với cách mạng.
+2. Sinh viên khuyết tật.
+3. Sinh viên từ 16 đến 22 tuổi mồ côi hoặc không nơi nương tựa đang hưởng trợ cấp xã hội hàng tháng.
+4. Sinh viên là người dân tộc thiểu số thuộc hộ nghèo hoặc hộ cận nghèo.
+5. Sinh viên dân tộc thiểu số rất ít người vùng khó khăn.</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>đối tượng miễn 100% học phí, Nghị định 81, con thương binh, dân tộc thiểu số</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="55" customHeight="1">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Đối tượng nào được giảm 70% học phí theo quy định?</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Sinh viên là người dân tộc thiểu số (không thuộc nhóm rất ít người) có hộ khẩu thường trú tại thôn/bản đặc biệt khó khăn, xã khu vực III vùng dân tộc và miền núi, xã đặc biệt khó khăn vùng bãi ngang ven biển hải đảo.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>giảm 70% học phí, vùng đặc biệt khó khăn, dân tộc thiểu số</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="55" customHeight="1">
+      <c r="A43" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Đối tượng nào được giảm 50% học phí?</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Sinh viên là con của cán bộ, công chức, viên chức, công nhân mà cha hoặc mẹ bị tai nạn lao động hoặc mắc bệnh nghề nghiệp được hưởng trợ cấp thường xuyên.</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>giảm 50% học phí, tai nạn lao động, bệnh nghề nghiệp</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="55" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Hồ sơ xin miễn giảm học phí gồm những giấy tờ gì?</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Hồ sơ gồm:
+1. Đơn xin miễn giảm học phí (theo mẫu của Trường).
+2. Bản sao có chứng thực giấy tờ chứng minh đối tượng (Giấy chứng nhận hộ nghèo/cận nghèo năm hiện hành, Thẻ thương binh, Giấy xác nhận khuyết tật...).
+3. Bản sao Giấy khai sinh và Căn cước công dân.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>hồ sơ miễn giảm học phí, giấy tờ cần nộp, mẫu đơn MGHP</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="55" customHeight="1">
+      <c r="A45" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Mức trợ cấp xã hội cho sinh viên mồ côi hoặc khuyết tật là bao nhiêu tiền 1 tháng?</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Mức trợ cấp xã hội là 100.000 đồng/sinh viên/tháng (riêng sinh viên dân tộc ít người thường trú ở vùng cao được 140.000 đồng/tháng), chi trả theo học kỳ.</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>trợ cấp xã hội, 100k một tháng, mồ côi, khuyết tật</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="55" customHeight="1">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Chính sách hỗ trợ chi phí học tập cho sinh viên dân tộc thiểu số nghèo được bao nhiêu tiền?</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Theo Thông tư liên tịch 35/2014, sinh viên dân tộc thiểu số thuộc hộ nghèo/cận nghèo được hỗ trợ 60% mức lương cơ sở/tháng x 10 tháng/năm học.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>hỗ trợ chi phí học tập, dân tộc thiểu số nghèo, 60% lương cơ sở</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="55" customHeight="1">
+      <c r="A47" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Chính sách hỗ trợ cho sinh viên dân tộc thiểu số rất ít người là bao nhiêu?</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Theo Nghị định 57/2017/NĐ-CP, sinh viên thuộc 16 dân tộc thiểu số rất ít người (Cống, Mảng, Pu Péo, Si La...) được hưởng hỗ trợ bằng 100% mức lương cơ sở x 12 tháng/năm học.</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>dân tộc thiểu số rất ít người, 100% lương cơ sở, Nghị định 57</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="55" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Sinh viên khuyết tật được hỗ trợ mua phương tiện học tập bao nhiêu tiền 1 năm?</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Theo Thông tư 42/2013, ngoài học bổng 80% lương cơ sở/tháng, sinh viên khuyết tật nghèo/cận nghèo còn được hỗ trợ 1.000.000 đồng/người/năm học để mua sắm phương tiện, đồ dùng học tập.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>sinh viên khuyết tật, hỗ trợ 1 triệu, đồ dùng học tập</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="55" customHeight="1">
+      <c r="A49" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Hồ sơ miễn giảm học phí có phải nộp lại mỗi năm không?</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>CÓ. Đối với diện hộ nghèo/cận nghèo, do sổ hộ nghèo chỉ có giá trị theo từng năm nên sinh viên bắt buộc phải nộp Giấy chứng nhận hộ nghèo mới vào đầu mỗi năm học. Đối với diện người có công hoặc khuyết tật chỉ cần nộp 1 lần cho cả khóa trừ khi có thông báo mới.</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>nộp lại mỗi năm, hiệu lực sổ hộ nghèo, giấy tờ hàng năm</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Thời gian xét học bổng tài trợ doanh nghiệp diễn ra khi nào?</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Các nguồn học bổng tài trợ từ doanh nghiệp, cựu sinh viên, tổ chức phi chính phủ được Phòng CTSV thông báo và xét chọn định kỳ từ tháng 9/2025 đến tháng 12/2025.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>học bổng tài trợ, thời gian xét học bổng, doanh nghiệp tài trợ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="55" customHeight="1">
+      <c r="A51" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Miễn giảm học phí</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên thuộc diện miễn giảm học phí có phải đóng học phí trước rồi nhận lại không?</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Tùy theo thông báo cụ thể của từng kỳ: Nếu hồ sơ được phê duyệt trước hạn đóng học phí thì sinh viên được trừ trực tiếp; nếu hồ sơ xét duyệt sau thì sinh viên đóng học phí tạm ứng và Nhà trường sẽ hoàn trả lại qua tài khoản ngân hàng sau khi có quyết định chính thức.</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>trừ học phí, hoàn trả tiền học phí, tạm ứng</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="55" customHeight="1">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Thời hạn xác nhận ngoại trú Học kỳ 1 năm học 2025-2026 là khi nào?</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Thời hạn xác nhận thông tin ngoại trú HK1 là từ ngày 27/10/2025 đến hết ngày 07/11/2025.</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>xác nhận ngoại trú, thời hạn ngoại trú, 27/10 đến 07/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="55" customHeight="1">
+      <c r="A53" s="5" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Không xác nhận ngoại trú đúng hạn bị xử lý kỷ luật thế nào?</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Sinh viên không khai báo hoặc không xác nhận ngoại trú đúng thời hạn sẽ BỊ TRỪ 15 ĐIỂM RÈN LUYỆN trong học kỳ tương ứng. Đây là mức phạt rất nặng làm mất xếp loại rèn luyện Tốt/Xuất sắc và mất học bổng.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>trừ 15 điểm rèn luyện, phạt ngoại trú, không xác nhận</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="55" customHeight="1">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Xác nhận ngoại trú thực hiện theo hình thức nào?</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Sinh viên thực hiện trực tuyến qua Cổng quản lý sinh viên của Trường hoặc nộp Giấy xác nhận tạm trú có xác nhận đóng dấu của Công an Phường/Xã nơi thuê trọ về Phòng Công tác Sinh viên.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>cách xác nhận ngoại trú, nộp giấy tạm trú, công an phường</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="55" customHeight="1">
+      <c r="A55" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên ở Ký túc xá ĐHQG-HCM có cần làm thủ tục xác nhận ngoại trú không?</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG. Sinh viên nội trú tại Ký túc xá ĐHQG-HCM hoặc KTX Trường sẽ được Ban Quản lý KTX lập danh sách đồng bộ trực tiếp với Phòng CTSV, sinh viên không cần làm xác nhận ngoại trú riêng.</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>ở KTX có cần xác nhận ngoại trú không, danh sách đồng bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="55" customHeight="1">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Nếu thay đổi chỗ trọ trong năm học thì phải báo trong thời gian bao lâu?</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Theo Quy chế Ngoại trú, khi thay đổi địa chỉ tạm trú, trong vòng 15 ngày làm việc sinh viên phải cập nhật lại thông tin địa chỉ mới trên hệ thống của Trường hoặc báo về Phòng CTSV.</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>đổi chỗ trọ, thay đổi địa chỉ ngoại trú, 15 ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="55" customHeight="1">
+      <c r="A57" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Phòng ban nào chịu trách nhiệm quản lý thông tin ngoại trú của sinh viên?</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Phòng Công tác Sinh viên (P. CTSV) là đơn vị đầu mối phụ trách tiếp nhận, quản lý và kiểm tra dữ liệu ngoại trú của sinh viên.</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>phòng quản lý ngoại trú, phòng CTSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Số điện thoại của Ký túc xá 135B Trần Hưng Đạo (Quận 5) là gì?</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Số điện thoại liên hệ KTX 135B Trần Hưng Đạo, Quận 5: (028) 38368670.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>KTX 135B Trần Hưng Đạo, số điện thoại KTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="55" customHeight="1">
+      <c r="A59" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Tổng đài hỗ trợ sinh viên của Trung tâm Quản lý KTX ĐHQG-HCM là số mấy?</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Tổng đài hỗ trợ sinh viên KTX ĐHQG-HCM: 1900.05.55.59 (nhánh lẻ 111 hoặc 114).</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>tổng đài KTX ĐHQG, 1900055559</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="55" customHeight="1">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Công an Phường Đông Hòa (khu vực Cơ sở 2 và KTX khu B) nằm ở đâu?</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Công an Phường Đông Hòa nằm trên Đường Trần Hưng Đạo (ngã ba Cây Lơn), Phường Đông Hòa, TP. Dĩ An (giáp ranh Khu ĐT ĐHQG-HCM).</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>công an phường Đông Hòa, tạm trú cơ sở 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="55" customHeight="1">
+      <c r="A61" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Ngoại trú &amp; Nội trú</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên ở cùng gia đình tại TP.HCM có phải khai báo ngoại trú không?</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>CÓ. Tất cả sinh viên không ở KTX đều phải khai báo địa chỉ cư trú thực tế của mình (kể cả nhà riêng hoặc nhà người thân) để Nhà trường quản lý thông tin liên lạc khi cần thiết.</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>ở nhà riêng có khai báo ngoại trú không, địa chỉ cư trú</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="55" customHeight="1">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Quá hạn đóng học phí thì bị xử lý thế nào?</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Theo Điểm a Khoản 2 Điều 16 Quy chế Đào tạo, sinh viên không hoàn thành nghĩa vụ nộp học phí đúng thời hạn quy định của Trường sẽ bị BUỘC THÔI HỌC VÀ XÓA TÊN KHỎI DANH SÁCH SINH VIÊN.</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>quá hạn học phí, buộc thôi học học phí, nợ học phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="55" customHeight="1">
+      <c r="A63" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Tôi có thể nộp học phí bằng những hình thức nào?</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Sinh viên nộp học phí trực tuyến qua cổng thanh toán liên kết ngân hàng của HCMUS (hướng dẫn trên Portal) hoặc nộp trực tiếp tại Phòng Kế hoạch Tài chính (Phòng B.01 Cơ sở 1 hoặc Phòng 2.7 Cơ sở 2).</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>cách đóng học phí, thanh toán trực tuyến, phòng kế hoạch tài chính</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="55" customHeight="1">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Nếu gia đình gặp khó khăn đột xuất chưa thể đóng học phí đúng hạn thì phải làm gì?</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Sinh viên phải làm 'Đơn xin gia hạn đóng học phí' (nêu rõ hoàn cảnh, có xác nhận của phụ huynh/địa phương và cam kết ngày đóng) nộp về Phòng CTSV TRƯỚC ngày hết hạn để được Ban Giám hiệu xem xét tạm hoãn nghĩa vụ.</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>xin gia hạn học phí, đơn hoãn học phí, khó khăn tài chính</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="55" customHeight="1">
+      <c r="A65" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Số điện thoại kiểm tra xác nhận đã hoàn tất đóng học phí là số nào?</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Liên hệ Phòng Kế hoạch Tài chính: Điện thoại (028) 38355275 hoặc (028) 62884499 (ext 1103); Email: taivu.khtn@gmail.com.</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>kiểm tra học phí, xác nhận đóng học phí, ext 1103, taivu.khtn</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="55" customHeight="1">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Sinh viên bị buộc thôi học do nợ học phí thì kết quả học tập trước đó có bị hủy không?</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Theo Khoản 4 Điều 16 Quy chế Đào tạo, kết quả học tập đã tích lũy của sinh viên trong trường hợp bị buộc thôi học vẫn được lưu trữ tại Trường để có thể công nhận chuyển đổi nếu học lại sau này.</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>bảo lưu điểm khi thôi học, kết quả học tập nợ học phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="55" customHeight="1">
+      <c r="A67" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Học phí học lại môn học được tính thế nào?</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Học phí học lại được tính dựa trên số tín chỉ của học phần đó nhân với đơn giá tín chỉ tương ứng của khóa học và hệ đào tạo theo quy định hiện hành của Trường.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>học phí học lại, tính tiền tín chỉ, đơn giá tín chỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="55" customHeight="1">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Học phần điểm I (hoãn thi) khi học lại có phải đóng học phí không?</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>KHÔNG. Theo Khoản 3 Điều 12 Quy chế Đào tạo, sinh viên đăng ký học lại học phần được nhận điểm I trong vòng 01 năm học tiếp theo sẽ KHÔNG PHẢI ĐÓNG HỌC PHÍ cho học phần này.</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>điểm I có đóng học phí không, miễn học phí điểm I</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="55" customHeight="1">
+      <c r="A69" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Thời hạn Nhà trường ra quyết định buộc thôi học đối với sinh viên nợ học phí?</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Theo Khoản 3 Điều 16, Nhà trường sẽ thông báo cho sinh viên biết chậm nhất 01 tháng sau khi có quyết định buộc thôi học.</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>thời hạn quyết định thôi học, 1 tháng</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="55" customHeight="1">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Sinh viên nợ học phí có được thi kết thúc học phần không?</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Theo quy định, sinh viên chưa hoàn thành nghĩa vụ học phí của học kỳ có thể bị khóa quyền xem lịch thi hoặc bị từ chối công nhận kết quả thi kết thúc học phần.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>nợ học phí có được thi không, cấm thi vì nợ học phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="55" customHeight="1">
+      <c r="A71" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Học phí &amp; Kỷ luật</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên có được rút học phí nếu xin nghỉ học giữa chừng không?</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Việc rút hoặc hoàn trả học phí được thực hiện theo Quy chế Tài chính của Trường, chỉ xem xét đối với các trường hợp rút học phần hợp lệ trong thời gian quy định đầu kỳ hoặc có lý do bất khả kháng được Hiệu trưởng phê duyệt.</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>rút học phí, hoàn trả học phí, nghỉ học rút tiền</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="55" customHeight="1">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Sinh viên Chương trình Chuẩn phải đăng ký tối thiểu bao nhiêu tín chỉ một học kỳ chính?</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Theo Điểm a Khoản 2 Điều 7 Quy chế Đào tạo, sinh viên hệ chuẩn phải đăng ký TỐI THIỂU 14 TÍN CHỈ trong học kỳ chính (không kể các môn GDQP, GDTC và Ngoại ngữ tổng quát).</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>tối thiểu 14 tín chỉ, khối chuẩn, quy định đăng ký môn</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="55" customHeight="1">
+      <c r="A73" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên Chương trình Chuẩn được đăng ký tối đa bao nhiêu tín chỉ một kỳ?</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Theo Điểm b Khoản 2 Điều 7, số tín chỉ đăng ký học TỐI ĐA trong một học kỳ chính đối với khối Chuẩn là 25 TÍN CHỈ; tối đa trong học kỳ hè là 12 TÍN CHỈ.</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>tối đa 25 tín chỉ, học kỳ hè tối đa 12 tín chỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="55" customHeight="1">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Sinh viên Chương trình Đề án (CLC/Tiên tiến) quy định số tín chỉ tối thiểu và tối đa thế nào?</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>- Tối thiểu: 10 TÍN CHỈ trong một học kỳ chính.
+- Tối đa: 22 TÍN CHỈ trong một học kỳ chính.</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>tín chỉ khối đề án, tối thiểu 10 tín chỉ, tối đa 22 tín chỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="55" customHeight="1">
+      <c r="A75" s="5" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên học cùng lúc hai chương trình (song bằng) được đăng ký tối đa bao nhiêu tín chỉ?</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>Theo Điểm c Khoản 2 Điều 7, sinh viên học cùng lúc hai chương trình được đăng ký TỐI ĐA 37 TÍN CHỈ trong mỗi học kỳ chính và không vượt quá 15 TÍN CHỈ trong học kỳ hè.</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>song bằng, học 2 chương trình, tối đa 37 tín chỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="55" customHeight="1">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Đã đăng ký học phần nhưng tự ý không đi học thì bị xử lý thế nào?</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Theo Điểm d Khoản 1 Điều 7, sinh viên không tham gia học học phần đã đăng ký được xem như TỰ Ý BỎ HỌC VÀ PHẢI NHẬN ĐIỂM 0 (không điểm). Nếu tự ý bỏ học từ 1 kỳ chính trở lên sẽ bị BUỘC THÔI HỌC.</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>bỏ học sau đăng ký, nhận điểm 0, tự ý bỏ học</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="55" customHeight="1">
+      <c r="A77" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Thế nào là 'Học phần tiên quyết'?</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Học phần tiên quyết đối với học phần A là học phần mà sinh viên BẮT BUỘC PHẢI HỌC VÀ THI ĐẠT (điểm &gt;= 5.0) mới được phép đăng ký học phần A.</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>học phần tiên quyết, điều kiện tiên quyết, thi đạt</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="55" customHeight="1">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Thế nào là 'Học phần học trước'?</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Học phần học trước đối với học phần A là học phần mà sinh viên chỉ cần HOÀN THÀNH QUÁ TRÌNH HỌC TẬP (đã tham gia học, có điểm quá trình/thi) trước khi đăng ký học phần A, không bắt buộc phải thi đạt.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>học phần học trước, phân biệt tiên quyết</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="55" customHeight="1">
+      <c r="A79" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Thế nào là 'Học phần song hành'?</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Hai học phần là song hành khi sinh viên đăng ký học phần này thì BẮT BUỘC ĐỒNG THỜI PHẢI ĐĂNG KÝ học phần kia trong cùng một học kỳ (thường là lý thuyết và thực hành đi kèm).</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>học phần song hành, đăng ký cùng lúc</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="55" customHeight="1">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Muốn đăng ký vượt quá số tín chỉ tối đa hoặc ít hơn số tín chỉ tối thiểu phải làm gì?</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Sinh viên phải làm Đơn đề nghị, có ý kiến đồng ý của Ban Chủ nhiệm Khoa và phải được HIỆU TRƯỞNG CHẤP THUẬN bằng văn bản.</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>xin vượt tín chỉ, dưới tín chỉ tối thiểu, đơn xin phép</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="55" customHeight="1">
+      <c r="A81" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Đăng ký học phần</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Một tín chỉ được quy đổi tương đương với bao nhiêu tiết học?</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Theo Khoản 3 Điều 3 Quy chế Đào tạo: 1 tín chỉ = 15 tiết học lý thuyết; hoặc 30 – 45 tiết thực hành/thí nghiệm; hoặc 30 tiết làm tiểu luận/đồ án/khóa luận tốt nghiệp (1 tiết = 50 phút).</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>quy đổi tín chỉ, 1 tín chỉ bằng bao nhiêu tiết, 15 tiết lý thuyết</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="55" customHeight="1">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện để được xem xét hoãn thi cuối kỳ là gì?</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Theo Khoản 1 Điều 12 Quy chế Đào tạo, sinh viên gặp các trường hợp đột xuất và có lý do chính đáng: ốm đau nằm viện, tai nạn, hoàn cảnh gia đình khó khăn đột xuất không thể dự thi kết thúc học phần.</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>điều kiện hoãn thi, lý do hoãn thi, ốm đau tai nạn</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="55" customHeight="1">
+      <c r="A83" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Thời hạn nộp đơn xin hoãn thi là bao lâu kể từ ngày thi?</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Theo Khoản 2 Điều 12, sinh viên phải hoàn tất học phí và nộp Đơn xin hoãn thi kèm giấy tờ xác nhận y tế hợp lệ về Phòng Đào tạo TRONG VÒNG 05 NGÀY LÀM VIỆC kể từ ngày thi của môn đó.</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>hạn nộp đơn hoãn thi, 05 ngày làm việc, nộp ở phòng đào tạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="55" customHeight="1">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Điểm của môn hoãn thi được ghi nhận thế nào trên bảng điểm?</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Học phần được chấp thuận hoãn thi sẽ được ghi nhận ký hiệu là ĐIỂM I (Incomplete). Sinh viên không bị điểm 0 trong học kỳ đó.</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>điểm I, ký hiệu điểm I, hoãn thi ghi điểm gì</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="55" customHeight="1">
+      <c r="A85" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Sau khi nhận điểm I, sinh viên phải hoàn thành môn đó trong thời hạn bao lâu?</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Sinh viên có trách nhiệm nộp đơn đăng ký học lại học phần hoãn thi TRONG VÒNG 01 NĂM HỌC TIẾP THEO. Khi học lại, sinh viên KHÔNG PHẢI ĐÓNG HỌC PHÍ.</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>trả nợ điểm I, thời hạn 1 năm, không đóng học phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="55" customHeight="1">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Điểm thành phần quá trình của môn hoãn thi có được bảo lưu không?</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>KHÔNG. Theo Khoản 4 Điều 12, điểm thành phần quá trình của học phần hoãn thi SẼ KHÔNG ĐƯỢC BẢO LƯU. Khi học lại, sinh viên phải làm lại bài tập, kiểm tra quá trình từ đầu.</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>bảo lưu điểm quá trình, điểm I có bảo lưu không</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="55" customHeight="1">
+      <c r="A87" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Học phần bắt buộc bị điểm dưới 5.0 thì xử lý thế nào?</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Theo Khoản 1 Điều 14, sinh viên có điểm học phần dưới 5.0 (không đạt) BẮT BUỘC PHẢI ĐĂNG KÝ HỌC LẠI học phần đó. Điểm lần học cuối là điểm chính thức của học phần.</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>học lại môn bắt buộc, dưới 5 điểm, điểm lần học cuối</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="55" customHeight="1">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Học phần tự chọn bị rớt (dưới 5.0) có bắt buộc phải học lại đúng môn đó không?</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Theo Điểm c Khoản 1 Điều 14, sinh viên được phép đăng ký học lại chính môn đó HOẶC chọn học một học phần tự chọn khác tương đương trong chương trình đào tạo để bù đủ tín chỉ.</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>rớt môn tự chọn, học môn khác thay thế</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="55" customHeight="1">
+      <c r="A89" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>Quy định về học cải thiện điểm như thế nào?</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>Theo Khoản 2 Điều 14, học phần đã đạt (&gt;= 5.0) nhưng sinh viên muốn nâng điểm thì đăng ký học lại và nộp học phí. Điểm lần học cuối là điểm chính thức (kể cả khi điểm mới thấp hơn điểm cũ).</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>học cải thiện điểm, nâng điểm, điểm lần cuối chính thức</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="55" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Điểm học cải thiện có được dùng để xét học bổng khuyến khích học kỳ đó không?</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>KHÔNG. Theo Điểm c Khoản 2 Điều 14, điểm cải thiện KHÔNG ĐƯỢC SỬ DỤNG để tính điểm trung bình học kỳ xét học bổng khuyến khích học tập, nhưng được tính vào điểm trung bình tích lũy toàn khóa.</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>cải thiện điểm xét học bổng, không tính học bổng</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="55" customHeight="1">
+      <c r="A91" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Hoãn thi &amp; Cải thiện</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Nếu vắng buổi kiểm tra quá trình có lý do chính đáng thì giải quyết thế nào?</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>Theo Khoản 4 Điều 12, giảng viên phụ trách môn học sẽ chủ động sắp xếp cho sinh viên được kiểm tra bù vào thời điểm khác trước ngày thi kết thúc học phần.</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>kiểm tra bù, vắng kiểm tra quá trình, giảng viên xếp lịch</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="55" customHeight="1">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Phúc khảo bài thi</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Nộp đơn phúc khảo bài thi kết thúc học phần ở đâu?</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Nộp tại Phòng Khảo thí và Đảm bảo Chất lượng:
+- Cơ sở 1: Phòng B.04, 227 Nguyễn Văn Cừ, Q.5.
+- Cơ sở 2: Phòng 2.5, Tầng 2 Tòa nhà Điều hành, Khu ĐT ĐHQG-HCM.</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>địa chỉ nộp phúc khảo, phòng B.04, phòng khảo thí</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="55" customHeight="1">
+      <c r="A93" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Phúc khảo bài thi</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>Thời hạn nộp đơn phúc khảo là bao lâu sau khi biết điểm thi?</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>Trong vòng 07 đến 10 ngày làm việc kể từ ngày công bố điểm thi chính thức trên Cổng Portal Đào tạo (theo thông báo của Phòng Khảo thí).</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>thời hạn nộp phúc khảo, 7 đến 10 ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="55" customHeight="1">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Phúc khảo bài thi</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Bao lâu thì có kết quả chấm phúc khảo?</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Theo Điều 15 Quy định Khảo thí, kết quả chấm phúc khảo được công bố trong vòng 15 NGÀY LÀM VIỆC kể từ ngày hết hạn nhận đơn phúc khảo.</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>kết quả phúc khảo, 15 ngày làm việc</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="55" customHeight="1">
+      <c r="A95" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Phúc khảo bài thi</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Nếu điểm phúc khảo thấp hơn điểm ban đầu thì lấy điểm nào?</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>Theo quy chế khảo thí, điểm chấm phúc khảo là KẾT QUẢ CUỐI CÙNG của bài thi, kể cả trường hợp điểm mới thấp hơn điểm đã công bố ban đầu.</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>điểm phúc khảo thấp hơn, nguyên tắc điểm phúc khảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="55" customHeight="1">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Phúc khảo bài thi</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Có được phúc khảo bài kiểm tra giữa kỳ không?</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Bài kiểm tra giữa kỳ do Khoa/Bộ môn và giảng viên trực tiếp quản lý, sinh viên liên hệ trực tiếp giảng viên phụ trách môn học trong tuần học kế tiếp để được xem lại bài kiểm tra.</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>phúc khảo giữa kỳ, liên hệ giảng viên</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="55" customHeight="1">
+      <c r="A97" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Chuẩn Ngoại ngữ</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>Sinh viên hệ đại trà phải hoàn thành bao nhiêu học phần tiếng Anh?</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Sinh viên phải hoàn tất 04 học phần Anh văn (từ Anh văn 1 đến Anh văn 4, không tính học phần bổ túc đầu khóa). Sinh viên được miễn 4 học phần này nếu đã nộp chứng chỉ đạt chuẩn ngoại ngữ đầu ra.</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>4 học phần Anh văn, AV1 đến AV4, miễn học phần tiếng Anh</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="55" customHeight="1">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Chuẩn Ngoại ngữ</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện về tiếng Anh để được đăng ký học các môn chuyên ngành là gì?</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Sinh viên phải thỏa mãn một trong 3 điều kiện:
+1. Đã đạt chuẩn ngoại ngữ đầu ra.
+2. Đã hoàn tất 04 học phần Anh văn (AV1 – AV4).
+3. Đạt từ 5.0 điểm trở lên trong kỳ thi đánh giá trình độ tiếng Anh nội bộ do Trường tổ chức.</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>điều kiện học chuyên ngành, tiếng Anh chuyên ngành, 5.0 nội bộ</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="55" customHeight="1">
+      <c r="A99" s="5" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Chuẩn Ngoại ngữ</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>Chứng chỉ tiếng Anh nộp xét chuẩn đầu ra có thời hạn hiệu lực bao lâu?</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>- Chứng chỉ có ghi hạn: Phải còn hiệu lực tại thời điểm nộp hồ sơ.
+- Chứng chỉ không ghi hạn: Có giá trị trong vòng 02 NĂM kể từ ngày cấp đến ngày nộp hồ sơ xét đạt chuẩn.</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>hiệu lực chứng chỉ tiếng Anh, 2 năm, hạn chứng chỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="55" customHeight="1">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Chuẩn Ngoại ngữ</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Sinh viên ngành Công nghệ thông tin có được dùng bằng tiếng Nhật để ra trường không?</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>CÓ. Riêng chương trình tăng cường tiếng Anh ngành CNTT, chứng chỉ tiếng Nhật JLPT cấp độ N2 (do tổ chức được Bộ GD&amp;ĐT / ĐHQG công nhận cấp) cũng được xét đạt chuẩn ngoại ngữ đầu ra.</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>tiếng Nhật N2, JLPT N2, chuẩn đầu ra CNTT</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="55" customHeight="1">
+      <c r="A101" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Chuẩn Ngoại ngữ</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>Thời hạn nộp chứng chỉ ngoại ngữ để kịp xét tốt nghiệp là khi nào?</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>Sinh viên phải nộp chứng chỉ ngoại ngữ về Phòng Đào tạo TRƯỚC thời hạn nộp hồ sơ xét tốt nghiệp của từng đợt xét trong năm (Trường có 4 đợt xét tốt nghiệp hàng năm).</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="inlineStr">
+        <is>
+          <t>hạn nộp bằng tiếng Anh tốt nghiệp, xét tốt nghiệp</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="55" customHeight="1">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Tiết học &amp; Liên hệ</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Tiết 1 buổi sáng ở Cơ sở 1 và Cơ sở 2 bắt đầu lúc mấy giờ?</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>- Cơ sở 1 (227 Nguyễn Văn Cừ, Q.5): Tiết 1 bắt đầu lúc 06g40 sáng (kết thúc lúc 07g30).
+- Cơ sở 2 (Khu ĐT ĐHQG-HCM, Thủ Đức): Tiết 1 bắt đầu lúc 07g30 sáng (kết thúc lúc 08g20). Cơ sở 2 bắt đầu muộn hơn CS1 đúng 50 phút.</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>tiết 1 bắt đầu mấy giờ, 6h40, 7h30, giờ học cơ sở 1 và cơ sở 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="55" customHeight="1">
+      <c r="A103" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Tiết học &amp; Liên hệ</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
+          <t>Cơ sở 2 (Thủ Đức) có tổ chức dạy ca tối không?</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>KHÔNG. Tại Cơ sở 2 chỉ tổ chức học 10 tiết từ sáng đến chiều (kết thúc lúc 17g00). Ca tối (tiết 13 đến 15, từ 18g00 đến 20g30) chỉ tổ chức tại Cơ sở 1.</t>
+        </is>
+      </c>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
+          <t>ca tối cơ sở 2, học buổi tối thủ đức, không dạy ca tối</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="55" customHeight="1">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Tiết học &amp; Liên hệ</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Tuyến xe buýt nào chạy thẳng kết nối giữa Cơ sở 1 và Cơ sở 2?</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Tuyến xe buýt số 08 (Bến xe Quận 8 – Đại học Quốc gia) là tuyến huyết mạch đi ngang qua Cơ sở 1 (đường Nguyễn Văn Cừ) và chạy thẳng đến Cơ sở 2 (Khu Đô thị ĐHQG). Ngoài ra có tuyến số 53 xuất phát từ Lê Hồng Phong (gần CS1).</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>xe buýt số 08, tuyến xe buýt kết nối, xe buýt 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="55" customHeight="1">
+      <c r="A105" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Tiết học &amp; Liên hệ</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>Số điện thoại Tổ bảo vệ và ANTT tại Cơ sở 1 và Cơ sở 2 là gì?</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>- Tổ bảo vệ Cơ sở 1 (Nguyễn Văn Cừ): 028.38356472.
+- Tổ bảo vệ Cổng chính Cơ sở 2 (Thủ Đức): 0986.635.439; Tổ bảo vệ Nhà Điều hành: 0982.341.039.</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>số điện thoại bảo vệ, an ninh trật tự, hotline cơ sở 1 và cơ sở 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="55" customHeight="1">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Tiết học &amp; Liên hệ</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>Hotline hỗ trợ tâm lý và giảm căng thẳng thi cử của Trường là số nào?</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Bộ phận Tham vấn Tâm lý (PSY.US) thuộc Phòng CTSV:
+- Hotline / Zalo: 0918.207.126 hoặc 0366.812.741.
+- Email: hotrosuckhoetinhthan@hcmus.edu.vn.
+- Địa chỉ: Phòng F106A (Cơ sở 1) và Phòng C110 (Cơ sở 2). Hỗ trợ hoàn toàn miễn phí và bảo mật.</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>tham vấn tâm lý, hotline tâm lý, PSY.US, căng thẳng thi cử</t>
         </is>
       </c>
     </row>

</xml_diff>